<commit_message>
feat: add updateRpaFields operation and modify process progress fields logic
- Add new operation `updateRpaFields` to update RPA field options from Excel data
- Include new Excel document `Curso_do_Aluno-Elaw.xlsx` as data source
- Update existing Excel document `cogna-process-progress-fields.xlsx`
- Modify process progress fields service to remove unnecessary validation errors
- Change create-progress-progress-fields operation to update existing fields instead of deleting all
- Add npm scripts for new operation in both development and production environments
- Register new operation in main operations array
</commit_message>
<xml_diff>
--- a/documents/cogna-process-progress-fields.xlsx
+++ b/documents/cogna-process-progress-fields.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="fields" sheetId="1" state="visible" r:id="rId1"/>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>label</t>
   </si>
@@ -38,6 +38,15 @@
     <t>isMultipleField</t>
   </si>
   <si>
+    <t xml:space="preserve">Número do processo</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>CNJ</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tipo de andamento</t>
   </si>
   <si>
@@ -74,9 +83,6 @@
     <t>Responsável</t>
   </si>
   <si>
-    <t>text</t>
-  </si>
-  <si>
     <t>Endereço</t>
   </si>
   <si>
@@ -146,10 +152,19 @@
     <t xml:space="preserve">Agravo Regimental</t>
   </si>
   <si>
+    <t xml:space="preserve">Opção teste 1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Agravo de Despacho Denegatório de Resp</t>
   </si>
   <si>
+    <t xml:space="preserve">Nova opção para testes</t>
+  </si>
+  <si>
     <t xml:space="preserve">Agravo de Despacho Denegatório de Rext</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terceira só pra fazer valer</t>
   </si>
   <si>
     <t xml:space="preserve">Agravo de Instrumento</t>
@@ -397,7 +412,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -406,9 +421,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
@@ -425,7 +437,6 @@
     <xf fontId="1" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -963,16 +974,18 @@
       <c r="C2" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="D2" s="4"/>
+      <c r="D2" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" ht="14.25">
       <c r="A3" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C3" s="4" t="b">
         <v>1</v>
@@ -983,7 +996,7 @@
     </row>
     <row r="4" ht="14.25">
       <c r="A4" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>10</v>
@@ -997,189 +1010,187 @@
     </row>
     <row r="5" ht="14.25">
       <c r="A5" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C5" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D5" s="4"/>
-      <c r="E5" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C7" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
-      <c r="F7" s="4" t="b">
-        <v>0</v>
-      </c>
+      <c r="F7" s="4"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>7</v>
+        <v>17</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="C8" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D8" s="4"/>
-      <c r="E8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>16</v>
+        <v>14</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="C9" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F9" s="4"/>
     </row>
     <row r="10" ht="14.25">
       <c r="A10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="5" t="s">
         <v>18</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="C10" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F10" s="4"/>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>7</v>
       </c>
       <c r="C11" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D11" s="4"/>
       <c r="E11" s="4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F11" s="4"/>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C12" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
+      <c r="E12" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="F12" s="4"/>
     </row>
     <row r="13" ht="14.25">
       <c r="A13" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C13" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="4" t="b">
-        <v>0</v>
-      </c>
+      <c r="F13" s="4"/>
     </row>
     <row r="14" ht="14.25">
       <c r="A14" s="4" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C14" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D14" s="4"/>
-      <c r="E14" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="4" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="C15" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F15" s="4"/>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" s="4" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="C16" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D16" s="4"/>
       <c r="E16" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F16" s="4"/>
     </row>
@@ -1188,99 +1199,101 @@
         <v>24</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="C17" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
+      <c r="E17" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="F17" s="4"/>
     </row>
     <row r="18" ht="14.25">
       <c r="A18" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="C18" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
-      <c r="F18" s="4" t="b">
-        <v>0</v>
-      </c>
+      <c r="F18" s="4"/>
     </row>
     <row r="19" ht="14.25">
       <c r="A19" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>16</v>
+        <v>27</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="C19" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D19" s="4"/>
-      <c r="E19" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" ht="14.25">
       <c r="A20" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>23</v>
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="C20" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F20" s="4"/>
     </row>
     <row r="21" ht="14.25">
       <c r="A21" s="4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C21" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F21" s="4"/>
     </row>
     <row r="22" ht="14.25">
       <c r="A22" s="4" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C22" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
+      <c r="E22" s="4" t="s">
+        <v>27</v>
+      </c>
       <c r="F22" s="4"/>
     </row>
     <row r="23" ht="14.25">
       <c r="A23" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C23" s="4" t="b">
         <v>1</v>
@@ -1291,10 +1304,10 @@
     </row>
     <row r="24" ht="14.25">
       <c r="A24" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C24" s="4" t="b">
         <v>1</v>
@@ -1305,10 +1318,10 @@
     </row>
     <row r="25" ht="14.25">
       <c r="A25" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>16</v>
+        <v>30</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="C25" s="4" t="b">
         <v>1</v>
@@ -1319,10 +1332,10 @@
     </row>
     <row r="26" ht="14.25">
       <c r="A26" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>16</v>
+        <v>31</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>19</v>
       </c>
       <c r="C26" s="4" t="b">
         <v>1</v>
@@ -1333,17 +1346,15 @@
     </row>
     <row r="27" ht="14.25">
       <c r="A27" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C27" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>32</v>
-      </c>
+      <c r="D27" s="4"/>
       <c r="E27" s="4"/>
       <c r="F27" s="4"/>
     </row>
@@ -1352,36 +1363,36 @@
         <v>33</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C28" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="D28" s="4"/>
+      <c r="D28" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="E28" s="4"/>
-      <c r="F28" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="F28" s="4"/>
     </row>
     <row r="29" ht="14.25">
       <c r="A29" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C29" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D29" s="4"/>
-      <c r="E29" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="30" ht="14.25">
       <c r="A30" s="4" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>7</v>
@@ -1391,59 +1402,67 @@
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F30" s="4"/>
     </row>
     <row r="31" ht="14.25">
       <c r="A31" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C31" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C31" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="6"/>
+      <c r="F31" s="4"/>
     </row>
     <row r="32" ht="14.25">
       <c r="A32" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C32" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
-      <c r="F32" s="6"/>
+      <c r="F32" s="5"/>
     </row>
     <row r="33" ht="14.25">
       <c r="A33" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="C33" s="4" t="b">
         <v>1</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
-      <c r="F33" s="6"/>
+      <c r="F33" s="5"/>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
-      <c r="F34" s="7"/>
+      <c r="A34" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="5"/>
     </row>
     <row r="35" ht="14.25">
       <c r="A35" s="1"/>
@@ -1451,7 +1470,7 @@
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
-      <c r="F35" s="7"/>
+      <c r="F35" s="6"/>
     </row>
     <row r="36" ht="14.25">
       <c r="A36" s="1"/>
@@ -1459,7 +1478,7 @@
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
-      <c r="F36" s="7"/>
+      <c r="F36" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -1476,449 +1495,549 @@
     <col customWidth="1" min="1" max="1" style="1" width="54.57421875"/>
     <col customWidth="1" min="2" max="2" style="1" width="37.57421875"/>
     <col customWidth="1" min="3" max="3" style="1" width="37.140625"/>
-    <col customWidth="1" min="4" max="4" style="1" width="26.8515625"/>
+    <col customWidth="1" min="4" max="4" style="1" width="60.57421875"/>
     <col customWidth="1" min="5" max="5" style="1" width="26.57421875"/>
     <col min="6" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="1">
-      <c r="A1" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="E1" s="8" t="s">
+      <c r="A1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>40</v>
       </c>
+      <c r="D1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="s">
-        <v>41</v>
+      <c r="A2" s="8" t="s">
+        <v>43</v>
       </c>
       <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
+      <c r="C2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="E2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="s">
-        <v>42</v>
+      <c r="A3" s="8" t="s">
+        <v>45</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
+      <c r="C3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>45</v>
+      </c>
       <c r="E3" s="4"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="s">
-        <v>43</v>
+      <c r="A4" s="8" t="s">
+        <v>47</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
+      <c r="C4" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>47</v>
+      </c>
       <c r="E4" s="4"/>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="s">
-        <v>44</v>
+      <c r="A5" s="8" t="s">
+        <v>49</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
+      <c r="D5" s="8" t="s">
+        <v>49</v>
+      </c>
       <c r="E5" s="4"/>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="s">
-        <v>45</v>
+      <c r="A6" s="8" t="s">
+        <v>50</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
+      <c r="D6" s="8" t="s">
+        <v>50</v>
+      </c>
       <c r="E6" s="4"/>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="s">
-        <v>46</v>
+      <c r="A7" s="8" t="s">
+        <v>51</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
+      <c r="D7" s="8" t="s">
+        <v>51</v>
+      </c>
       <c r="E7" s="4"/>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="s">
-        <v>47</v>
+      <c r="A8" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
+      <c r="D8" s="8" t="s">
+        <v>52</v>
+      </c>
       <c r="E8" s="4"/>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="s">
-        <v>48</v>
+      <c r="A9" s="8" t="s">
+        <v>53</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="D9" s="8" t="s">
+        <v>53</v>
+      </c>
       <c r="E9" s="4"/>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="s">
-        <v>49</v>
+      <c r="A10" s="8" t="s">
+        <v>54</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
+      <c r="D10" s="8" t="s">
+        <v>54</v>
+      </c>
       <c r="E10" s="4"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="s">
-        <v>50</v>
+      <c r="A11" s="8" t="s">
+        <v>55</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="D11" s="8" t="s">
+        <v>55</v>
+      </c>
       <c r="E11" s="4"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="s">
-        <v>51</v>
+      <c r="A12" s="8" t="s">
+        <v>56</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
+      <c r="D12" s="8" t="s">
+        <v>56</v>
+      </c>
       <c r="E12" s="4"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="s">
-        <v>52</v>
+      <c r="A13" s="8" t="s">
+        <v>57</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+      <c r="D13" s="8" t="s">
+        <v>57</v>
+      </c>
       <c r="E13" s="4"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="s">
-        <v>53</v>
+      <c r="A14" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="B14" s="4"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
+      <c r="D14" s="8" t="s">
+        <v>58</v>
+      </c>
       <c r="E14" s="4"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="s">
-        <v>54</v>
+      <c r="A15" s="8" t="s">
+        <v>59</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
+      <c r="D15" s="8" t="s">
+        <v>59</v>
+      </c>
       <c r="E15" s="4"/>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="s">
-        <v>55</v>
+      <c r="A16" s="8" t="s">
+        <v>60</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
+      <c r="D16" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="E16" s="4"/>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="s">
-        <v>56</v>
+      <c r="A17" s="8" t="s">
+        <v>61</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
+      <c r="D17" s="8" t="s">
+        <v>61</v>
+      </c>
       <c r="E17" s="4"/>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="s">
-        <v>57</v>
+      <c r="A18" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
+      <c r="D18" s="8" t="s">
+        <v>62</v>
+      </c>
       <c r="E18" s="4"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="s">
-        <v>58</v>
+      <c r="A19" s="8" t="s">
+        <v>63</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
+      <c r="D19" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="E19" s="4"/>
     </row>
     <row r="20">
-      <c r="A20" s="9" t="s">
-        <v>59</v>
+      <c r="A20" s="8" t="s">
+        <v>64</v>
       </c>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
+      <c r="D20" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="E20" s="4"/>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="s">
-        <v>60</v>
+      <c r="A21" s="8" t="s">
+        <v>65</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
+      <c r="D21" s="8" t="s">
+        <v>65</v>
+      </c>
       <c r="E21" s="4"/>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="s">
-        <v>61</v>
+      <c r="A22" s="8" t="s">
+        <v>66</v>
       </c>
       <c r="B22" s="4"/>
       <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
+      <c r="D22" s="8" t="s">
+        <v>66</v>
+      </c>
       <c r="E22" s="4"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="s">
-        <v>62</v>
+      <c r="A23" s="8" t="s">
+        <v>67</v>
       </c>
       <c r="B23" s="4"/>
       <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
+      <c r="D23" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="E23" s="4"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="s">
-        <v>63</v>
+      <c r="A24" s="8" t="s">
+        <v>68</v>
       </c>
       <c r="B24" s="4"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
+      <c r="D24" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="E24" s="4"/>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="s">
-        <v>64</v>
+      <c r="A25" s="8" t="s">
+        <v>69</v>
       </c>
       <c r="B25" s="4"/>
       <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
+      <c r="D25" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="E25" s="4"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="s">
-        <v>65</v>
+      <c r="A26" s="8" t="s">
+        <v>70</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
+      <c r="D26" s="8" t="s">
+        <v>70</v>
+      </c>
       <c r="E26" s="4"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="s">
-        <v>66</v>
+      <c r="A27" s="8" t="s">
+        <v>71</v>
       </c>
       <c r="B27" s="4"/>
       <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
+      <c r="D27" s="8" t="s">
+        <v>71</v>
+      </c>
       <c r="E27" s="4"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="s">
-        <v>67</v>
+      <c r="A28" s="8" t="s">
+        <v>72</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
+      <c r="D28" s="8" t="s">
+        <v>72</v>
+      </c>
       <c r="E28" s="4"/>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="s">
-        <v>68</v>
+      <c r="A29" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="B29" s="4"/>
       <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
+      <c r="D29" s="8" t="s">
+        <v>73</v>
+      </c>
       <c r="E29" s="4"/>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="s">
-        <v>69</v>
+      <c r="A30" s="8" t="s">
+        <v>74</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
+      <c r="D30" s="8" t="s">
+        <v>74</v>
+      </c>
       <c r="E30" s="4"/>
     </row>
     <row r="31">
-      <c r="A31" s="9" t="s">
-        <v>70</v>
+      <c r="A31" s="8" t="s">
+        <v>75</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
+      <c r="D31" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="E31" s="4"/>
     </row>
     <row r="32">
-      <c r="A32" s="9" t="s">
-        <v>71</v>
+      <c r="A32" s="8" t="s">
+        <v>76</v>
       </c>
       <c r="B32" s="4"/>
       <c r="C32" s="4"/>
-      <c r="D32" s="4"/>
+      <c r="D32" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="E32" s="4"/>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="s">
-        <v>72</v>
+      <c r="A33" s="8" t="s">
+        <v>77</v>
       </c>
       <c r="B33" s="4"/>
       <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
+      <c r="D33" s="8" t="s">
+        <v>77</v>
+      </c>
       <c r="E33" s="4"/>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="s">
-        <v>73</v>
+      <c r="A34" s="8" t="s">
+        <v>78</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
+      <c r="D34" s="8" t="s">
+        <v>78</v>
+      </c>
       <c r="E34" s="4"/>
     </row>
     <row r="35">
-      <c r="A35" s="9" t="s">
-        <v>74</v>
+      <c r="A35" s="8" t="s">
+        <v>79</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
-      <c r="D35" s="4"/>
+      <c r="D35" s="8" t="s">
+        <v>79</v>
+      </c>
       <c r="E35" s="4"/>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="9" t="s">
-        <v>75</v>
+      <c r="A36" s="8" t="s">
+        <v>80</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
+      <c r="D36" s="8" t="s">
+        <v>80</v>
+      </c>
       <c r="E36" s="4"/>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="9" t="s">
-        <v>76</v>
+      <c r="A37" s="8" t="s">
+        <v>81</v>
       </c>
       <c r="B37" s="4"/>
       <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
+      <c r="D37" s="8" t="s">
+        <v>81</v>
+      </c>
       <c r="E37" s="4"/>
     </row>
     <row r="38" ht="14.25">
-      <c r="A38" s="9" t="s">
-        <v>77</v>
+      <c r="A38" s="8" t="s">
+        <v>82</v>
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
+      <c r="D38" s="8" t="s">
+        <v>82</v>
+      </c>
       <c r="E38" s="4"/>
     </row>
     <row r="39" ht="14.25">
-      <c r="A39" s="9" t="s">
-        <v>78</v>
+      <c r="A39" s="8" t="s">
+        <v>83</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
+      <c r="D39" s="8" t="s">
+        <v>83</v>
+      </c>
       <c r="E39" s="4"/>
     </row>
     <row r="40" ht="14.25">
-      <c r="A40" s="9" t="s">
-        <v>79</v>
+      <c r="A40" s="8" t="s">
+        <v>84</v>
       </c>
       <c r="B40" s="4"/>
       <c r="C40" s="4"/>
-      <c r="D40" s="4"/>
+      <c r="D40" s="8" t="s">
+        <v>84</v>
+      </c>
       <c r="E40" s="4"/>
     </row>
     <row r="41" ht="14.25">
-      <c r="A41" s="9" t="s">
-        <v>80</v>
+      <c r="A41" s="8" t="s">
+        <v>85</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
+      <c r="D41" s="8" t="s">
+        <v>85</v>
+      </c>
       <c r="E41" s="4"/>
     </row>
     <row r="42" ht="14.25">
-      <c r="A42" s="9" t="s">
-        <v>81</v>
+      <c r="A42" s="8" t="s">
+        <v>86</v>
       </c>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
-      <c r="D42" s="4"/>
+      <c r="D42" s="8" t="s">
+        <v>86</v>
+      </c>
       <c r="E42" s="4"/>
     </row>
     <row r="43" ht="14.25">
-      <c r="A43" s="9" t="s">
-        <v>82</v>
+      <c r="A43" s="8" t="s">
+        <v>87</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
+      <c r="D43" s="8" t="s">
+        <v>87</v>
+      </c>
       <c r="E43" s="4"/>
     </row>
     <row r="44" ht="14.25">
-      <c r="A44" s="9" t="s">
-        <v>83</v>
+      <c r="A44" s="8" t="s">
+        <v>88</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
-      <c r="D44" s="4"/>
+      <c r="D44" s="8" t="s">
+        <v>88</v>
+      </c>
       <c r="E44" s="4"/>
     </row>
     <row r="45" ht="14.25">
-      <c r="A45" s="9" t="s">
-        <v>84</v>
+      <c r="A45" s="8" t="s">
+        <v>89</v>
       </c>
       <c r="B45" s="4"/>
       <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
+      <c r="D45" s="8" t="s">
+        <v>89</v>
+      </c>
       <c r="E45" s="4"/>
     </row>
     <row r="46" ht="14.25">
-      <c r="A46" s="9" t="s">
-        <v>85</v>
+      <c r="A46" s="8" t="s">
+        <v>90</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
+      <c r="D46" s="8" t="s">
+        <v>90</v>
+      </c>
       <c r="E46" s="4"/>
     </row>
     <row r="47" ht="14.25">
-      <c r="A47" s="9" t="s">
-        <v>86</v>
+      <c r="A47" s="8" t="s">
+        <v>91</v>
       </c>
       <c r="B47" s="4"/>
       <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
+      <c r="D47" s="8" t="s">
+        <v>91</v>
+      </c>
       <c r="E47" s="4"/>
     </row>
     <row r="48" ht="14.25">
-      <c r="A48" s="9" t="s">
-        <v>87</v>
+      <c r="A48" s="8" t="s">
+        <v>92</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
-      <c r="D48" s="4"/>
+      <c r="D48" s="8" t="s">
+        <v>92</v>
+      </c>
       <c r="E48" s="4"/>
     </row>
   </sheetData>
@@ -1940,67 +2059,66 @@
   </cols>
   <sheetData>
     <row r="1" s="2" customFormat="1">
-      <c r="A1" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="B1" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>91</v>
+      <c r="A1" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D2" s="6"/>
+      <c r="A2" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="5"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D3" s="6"/>
+      <c r="A3" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D3" s="5"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="A4" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D4" s="5"/>
+    </row>
+    <row r="5" ht="14.25">
+      <c r="A5" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D4" s="6"/>
-    </row>
-    <row r="5" ht="14.25">
-      <c r="A5" s="11" t="s">
+      <c r="C5" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D5" s="6"/>
-      <c r="E5"/>
+      <c r="D5" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>